<commit_message>
updating the country calculation results
</commit_message>
<xml_diff>
--- a/personal/country-comparison-2026/Boss-Country-FIRE-Analysis.xlsx
+++ b/personal/country-comparison-2026/Boss-Country-FIRE-Analysis.xlsx
@@ -10,9 +10,9 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Save-By Targets" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Inputs" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Visa Pathways" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Hybrid Plans" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Visa Pathways" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Hybrid Plans" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Inputs" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Cost-of-Living" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Sensitivity" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="262">
   <si>
     <t xml:space="preserve">FIRE Calculator — Multi-Country Retirement Analysis</t>
   </si>
@@ -272,132 +272,6 @@
   </si>
   <si>
     <t xml:space="preserve">Notes: Real Portfolio is in TODAY's purchasing power. Nominal Book Value is what your broker statement will literally read in that year (after 3% inflation drift). Cushion = (Calc engine required) − (4% rule). Negative cushion is OK because Social Security at age 67 covers the gap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boss's RR Dashboard Baseline Parameters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Section</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roger age</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rebecca age</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kid 1 age</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kid 2 age</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plan to age</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Income</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annual income ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raise rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Effective tax rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portfolio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roger 401(k) Trad ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roger 401(k) Roth ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roger taxable ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rebecca taxable ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cash savings ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other assets ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL NET WORTH ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Returns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stock return (nominal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">401(k) return (nominal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inflation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real return (stocks)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contributions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monthly savings ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annual savings ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">401(k) Trad ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">401(k) Roth ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employer match ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL ANNUAL ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SS claim age</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SS COLA rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buffers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pre-unlock buffer (× spend)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SS-claim buffer (× spend)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Withdrawal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SWR (4% rule)</t>
   </si>
   <si>
     <t xml:space="preserve">Visa Pathways — Strategy by Country (May 2026, Updated)</t>
@@ -766,6 +640,9 @@
     <t xml:space="preserve">FASTEST FIRE. English-speaking beach base. Cheapest hybrid.</t>
   </si>
   <si>
+    <t xml:space="preserve">Hybrid: Japan + Indonesia/Bali (50/50)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Taiwan only</t>
   </si>
   <si>
@@ -803,6 +680,132 @@
   </si>
   <si>
     <t xml:space="preserve">• "End balance @ 100" is the surplus left in your portfolio at age 100, in TODAY's purchasing power.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boss's RR Dashboard Baseline Parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roger age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rebecca age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kid 1 age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kid 2 age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan to age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Income</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual income ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raise rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effective tax rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portfolio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roger 401(k) Trad ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roger 401(k) Roth ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roger taxable ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rebecca taxable ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash savings ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other assets ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL NET WORTH ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Returns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stock return (nominal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">401(k) return (nominal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inflation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real return (stocks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contributions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly savings ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual savings ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">401(k) Trad ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">401(k) Roth ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employer match ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL ANNUAL ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SS claim age</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SS COLA rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buffers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-unlock buffer (× spend)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SS-claim buffer (× spend)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Withdrawal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SWR (4% rule)</t>
   </si>
   <si>
     <t xml:space="preserve">2026 Upper-Middle-Class Cost of Living — Researched Monthly Breakdown</t>
@@ -1201,7 +1204,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1330,6 +1333,14 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1386,6 +1397,70 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1402,80 +1477,12 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2402,25 +2409,25 @@
         <v>48</v>
       </c>
       <c r="B12" s="15" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>66000</v>
+        <v>78000</v>
       </c>
       <c r="D12" s="17" t="n">
-        <v>1650000</v>
+        <v>1950000</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>1626620.94246088</v>
+        <v>1738381.78015932</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>2534222.42751448</v>
+        <v>2789592.43623367</v>
       </c>
       <c r="G12" s="20" t="n">
-        <v>-23379.057539118</v>
+        <v>-211618.219840683</v>
       </c>
       <c r="H12" s="21" t="n">
-        <v>-0.0141691257812836</v>
+        <v>-0.108522164020863</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2457,22 +2464,22 @@
         <v>57</v>
       </c>
       <c r="C14" s="26" t="n">
-        <v>57000</v>
+        <v>63000</v>
       </c>
       <c r="D14" s="27" t="n">
-        <v>1425000</v>
+        <v>1575000</v>
       </c>
       <c r="E14" s="28" t="n">
-        <v>1635620.94246088</v>
+        <v>1629620.94246088</v>
       </c>
       <c r="F14" s="29" t="n">
-        <v>2548244.13426389</v>
+        <v>2538896.32976428</v>
       </c>
       <c r="G14" s="30" t="n">
-        <v>210620.942460882</v>
+        <v>54620.942460882</v>
       </c>
       <c r="H14" s="31" t="n">
-        <v>0.147804170147987</v>
+        <v>0.0346799634672267</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2483,22 +2490,22 @@
         <v>57</v>
       </c>
       <c r="C15" s="26" t="n">
-        <v>60000</v>
+        <v>69000</v>
       </c>
       <c r="D15" s="27" t="n">
-        <v>1500000</v>
+        <v>1725000</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>1632620.94246088</v>
+        <v>1623620.94246088</v>
       </c>
       <c r="F15" s="29" t="n">
-        <v>2543570.23201409</v>
-      </c>
-      <c r="G15" s="30" t="n">
-        <v>132620.942460882</v>
-      </c>
-      <c r="H15" s="31" t="n">
-        <v>0.088413961640588</v>
+        <v>2529548.52526468</v>
+      </c>
+      <c r="G15" s="32" t="n">
+        <v>-101379.057539118</v>
+      </c>
+      <c r="H15" s="33" t="n">
+        <v>-0.0587704681386191</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2506,38 +2513,38 @@
         <v>52</v>
       </c>
       <c r="B16" s="25" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C16" s="26" t="n">
-        <v>51000</v>
+        <v>57000</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>1275000</v>
+        <v>1425000</v>
       </c>
       <c r="E16" s="28" t="n">
-        <v>1522620.13698162</v>
+        <v>1635620.94246088</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>2303099.57405588</v>
+        <v>2548244.13426389</v>
       </c>
       <c r="G16" s="30" t="n">
-        <v>247620.136981617</v>
+        <v>210620.942460882</v>
       </c>
       <c r="H16" s="31" t="n">
-        <v>0.194211872142445</v>
+        <v>0.147804170147987</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="32"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
@@ -2572,10 +2579,10 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="33" t="n">
+      <c r="A24" s="35" t="n">
         <v>42</v>
       </c>
-      <c r="B24" s="34" t="s">
+      <c r="B24" s="36" t="s">
         <v>60</v>
       </c>
       <c r="C24" s="18" t="n">
@@ -2584,18 +2591,18 @@
       <c r="D24" s="19" t="n">
         <v>473000</v>
       </c>
-      <c r="E24" s="35" t="s">
+      <c r="E24" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="36" t="s">
+      <c r="F24" s="38" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37" t="n">
+      <c r="A25" s="39" t="n">
         <v>49</v>
       </c>
-      <c r="B25" s="34" t="s">
+      <c r="B25" s="36" t="s">
         <v>63</v>
       </c>
       <c r="C25" s="18" t="n">
@@ -2604,18 +2611,18 @@
       <c r="D25" s="19" t="n">
         <v>1255000</v>
       </c>
-      <c r="E25" s="38" t="s">
+      <c r="E25" s="40" t="s">
         <v>64</v>
       </c>
-      <c r="F25" s="36" t="s">
+      <c r="F25" s="38" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="39" t="n">
+      <c r="A26" s="41" t="n">
         <v>53</v>
       </c>
-      <c r="B26" s="34" t="s">
+      <c r="B26" s="36" t="s">
         <v>66</v>
       </c>
       <c r="C26" s="18" t="n">
@@ -2624,18 +2631,18 @@
       <c r="D26" s="19" t="n">
         <v>1945000</v>
       </c>
-      <c r="E26" s="40" t="s">
+      <c r="E26" s="42" t="s">
         <v>67</v>
       </c>
-      <c r="F26" s="36" t="s">
+      <c r="F26" s="38" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="41" t="n">
+      <c r="A27" s="43" t="n">
         <v>55</v>
       </c>
-      <c r="B27" s="34" t="s">
+      <c r="B27" s="36" t="s">
         <v>69</v>
       </c>
       <c r="C27" s="18" t="n">
@@ -2644,18 +2651,18 @@
       <c r="D27" s="19" t="n">
         <v>2376000</v>
       </c>
-      <c r="E27" s="42" t="s">
+      <c r="E27" s="44" t="s">
         <v>70</v>
       </c>
-      <c r="F27" s="36" t="s">
+      <c r="F27" s="38" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="41" t="n">
+      <c r="A28" s="43" t="n">
         <v>57</v>
       </c>
-      <c r="B28" s="34" t="s">
+      <c r="B28" s="36" t="s">
         <v>72</v>
       </c>
       <c r="C28" s="18" t="n">
@@ -2664,18 +2671,18 @@
       <c r="D28" s="19" t="n">
         <v>2876000</v>
       </c>
-      <c r="E28" s="42" t="s">
+      <c r="E28" s="44" t="s">
         <v>73</v>
       </c>
-      <c r="F28" s="36" t="s">
+      <c r="F28" s="38" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="39" t="n">
+      <c r="A29" s="41" t="n">
         <v>59</v>
       </c>
-      <c r="B29" s="34" t="s">
+      <c r="B29" s="36" t="s">
         <v>75</v>
       </c>
       <c r="C29" s="18" t="n">
@@ -2684,18 +2691,18 @@
       <c r="D29" s="19" t="n">
         <v>3465000</v>
       </c>
-      <c r="E29" s="40" t="s">
+      <c r="E29" s="42" t="s">
         <v>76</v>
       </c>
-      <c r="F29" s="36" t="s">
+      <c r="F29" s="38" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="43" t="n">
+      <c r="A30" s="45" t="n">
         <v>61</v>
       </c>
-      <c r="B30" s="34" t="s">
+      <c r="B30" s="36" t="s">
         <v>78</v>
       </c>
       <c r="C30" s="18" t="n">
@@ -2704,24 +2711,24 @@
       <c r="D30" s="19" t="n">
         <v>3817000</v>
       </c>
-      <c r="E30" s="44" t="s">
+      <c r="E30" s="46" t="s">
         <v>79</v>
       </c>
-      <c r="F30" s="36" t="s">
+      <c r="F30" s="38" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="45" t="s">
+      <c r="A33" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="B33" s="45"/>
-      <c r="C33" s="45"/>
-      <c r="D33" s="45"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="45"/>
-      <c r="G33" s="45"/>
-      <c r="H33" s="45"/>
+      <c r="B33" s="47"/>
+      <c r="C33" s="47"/>
+      <c r="D33" s="47"/>
+      <c r="E33" s="47"/>
+      <c r="F33" s="47"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2746,889 +2753,514 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="46" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="47" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="48" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="47" t="s">
-        <v>86</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C5" s="48" t="n">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="47" t="s">
-        <v>86</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="C6" s="48" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="47" t="s">
-        <v>86</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" s="48" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="47" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C8" s="48" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="47" t="s">
-        <v>92</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="47" t="s">
-        <v>92</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="C10" s="49" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="47" t="s">
-        <v>92</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="C11" s="49" t="n">
-        <v>0.28</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C12" s="8" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>58000</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>190000</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="C15" s="8" t="n">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="C18" s="8" t="n">
-        <v>473000</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="47" t="s">
-        <v>104</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="C19" s="49" t="n">
-        <v>0.07</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="47" t="s">
-        <v>104</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C20" s="49" t="n">
-        <v>0.07</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="47" t="s">
-        <v>104</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C21" s="49" t="n">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="47" t="s">
-        <v>104</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C22" s="49" t="n">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="47" t="s">
-        <v>109</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C23" s="8" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="47" t="s">
-        <v>109</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="C24" s="8" t="n">
-        <v>24000</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="47" t="s">
-        <v>109</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C25" s="8" t="n">
-        <v>8550</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="47" t="s">
-        <v>109</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C26" s="8" t="n">
-        <v>2850</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="47" t="s">
-        <v>109</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C27" s="8" t="n">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="47" t="s">
-        <v>109</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="C28" s="8" t="n">
-        <v>42600</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="47" t="s">
-        <v>116</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="C29" s="48" t="n">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="47" t="s">
-        <v>116</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="C30" s="49" t="n">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="47" t="s">
-        <v>119</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="C31" s="48" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="47" t="s">
-        <v>119</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="C32" s="48" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="47" t="s">
-        <v>122</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="C33" s="49" t="n">
-        <v>0.04</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
   <dimension ref="A1:I27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="50" t="s">
+        <v>93</v>
+      </c>
+      <c r="E5" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="F5" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="G5" s="50" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" s="50" t="s">
+        <v>97</v>
+      </c>
+      <c r="I5" s="50" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="49" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="50" t="s">
+        <v>100</v>
+      </c>
+      <c r="E6" s="50" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" s="50" t="s">
+        <v>102</v>
+      </c>
+      <c r="G6" s="50" t="s">
+        <v>103</v>
+      </c>
+      <c r="H6" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="I6" s="50" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="50" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="50" t="s">
+        <v>108</v>
+      </c>
+      <c r="F7" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="G7" s="50" t="s">
+        <v>110</v>
+      </c>
+      <c r="H7" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="I7" s="50" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" s="50" t="s">
+        <v>113</v>
+      </c>
+      <c r="E8" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="F8" s="50" t="s">
+        <v>115</v>
+      </c>
+      <c r="G8" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="H8" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="I8" s="50" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="50" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" s="50" t="s">
+        <v>120</v>
+      </c>
+      <c r="F9" s="50" t="s">
+        <v>121</v>
+      </c>
+      <c r="G9" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="H9" s="50" t="s">
+        <v>123</v>
+      </c>
+      <c r="I9" s="50" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="48" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>125</v>
+      </c>
+      <c r="D10" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="E10" s="50" t="s">
         <v>127</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="F10" s="50" t="s">
         <v>128</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="G10" s="50" t="s">
         <v>129</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="H10" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="I10" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="H4" s="13" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="48" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="49" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="D11" s="50" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="50" t="n">
+      <c r="E11" s="50" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" s="50" t="s">
+        <v>135</v>
+      </c>
+      <c r="G11" s="50" t="s">
+        <v>136</v>
+      </c>
+      <c r="H11" s="50" t="s">
+        <v>137</v>
+      </c>
+      <c r="I11" s="50" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="45" t="s">
+        <v>139</v>
+      </c>
+      <c r="D12" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="E12" s="50" t="s">
+        <v>134</v>
+      </c>
+      <c r="F12" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="G12" s="50" t="s">
+        <v>142</v>
+      </c>
+      <c r="H12" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="I12" s="50" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="48" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="45" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13" s="50" t="s">
+        <v>145</v>
+      </c>
+      <c r="E13" s="50" t="s">
+        <v>134</v>
+      </c>
+      <c r="F13" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="G13" s="50" t="s">
+        <v>147</v>
+      </c>
+      <c r="H13" s="50" t="s">
+        <v>148</v>
+      </c>
+      <c r="I13" s="50" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="34"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="51" t="s">
+      <c r="B19" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="D5" s="52" t="s">
-        <v>135</v>
-      </c>
-      <c r="E5" s="52" t="s">
-        <v>136</v>
-      </c>
-      <c r="F5" s="52" t="s">
-        <v>137</v>
-      </c>
-      <c r="G5" s="52" t="s">
-        <v>138</v>
-      </c>
-      <c r="H5" s="52" t="s">
-        <v>139</v>
-      </c>
-      <c r="I5" s="52" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="50" t="n">
+      <c r="C19" s="50" t="s">
+        <v>154</v>
+      </c>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="54"/>
+      <c r="G19" s="54"/>
+      <c r="H19" s="54"/>
+      <c r="I19" s="54"/>
+    </row>
+    <row r="20" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="51" t="s">
-        <v>141</v>
-      </c>
-      <c r="C6" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="D6" s="52" t="s">
-        <v>142</v>
-      </c>
-      <c r="E6" s="52" t="s">
-        <v>143</v>
-      </c>
-      <c r="F6" s="52" t="s">
-        <v>144</v>
-      </c>
-      <c r="G6" s="52" t="s">
-        <v>145</v>
-      </c>
-      <c r="H6" s="52" t="s">
-        <v>146</v>
-      </c>
-      <c r="I6" s="52" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="50" t="n">
+      <c r="B20" s="49" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="50" t="s">
+        <v>155</v>
+      </c>
+      <c r="D20" s="50"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="54"/>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="54"/>
+    </row>
+    <row r="21" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="48" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="51" t="s">
+      <c r="B21" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="53" t="s">
-        <v>148</v>
-      </c>
-      <c r="D7" s="52" t="s">
-        <v>149</v>
-      </c>
-      <c r="E7" s="52" t="s">
-        <v>150</v>
-      </c>
-      <c r="F7" s="52" t="s">
-        <v>151</v>
-      </c>
-      <c r="G7" s="52" t="s">
-        <v>152</v>
-      </c>
-      <c r="H7" s="52" t="s">
-        <v>153</v>
-      </c>
-      <c r="I7" s="52" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="50" t="n">
+      <c r="C21" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="D21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="54"/>
+      <c r="G21" s="54"/>
+      <c r="H21" s="54"/>
+      <c r="I21" s="54"/>
+    </row>
+    <row r="22" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="48" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="51" t="s">
+      <c r="B22" s="49" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="53" t="s">
-        <v>148</v>
-      </c>
-      <c r="D8" s="52" t="s">
-        <v>155</v>
-      </c>
-      <c r="E8" s="52" t="s">
-        <v>156</v>
-      </c>
-      <c r="F8" s="52" t="s">
+      <c r="C22" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="G8" s="52" t="s">
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="54"/>
+      <c r="G22" s="54"/>
+      <c r="H22" s="54"/>
+      <c r="I22" s="54"/>
+    </row>
+    <row r="23" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="50" t="s">
         <v>158</v>
       </c>
-      <c r="H8" s="52" t="s">
+      <c r="D23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="54"/>
+      <c r="G23" s="54"/>
+      <c r="H23" s="54"/>
+      <c r="I23" s="54"/>
+    </row>
+    <row r="24" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="48" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="50" t="s">
         <v>159</v>
       </c>
-      <c r="I8" s="52" t="s">
+      <c r="D24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="54"/>
+      <c r="G24" s="54"/>
+      <c r="H24" s="54"/>
+      <c r="I24" s="54"/>
+    </row>
+    <row r="25" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="48" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="49" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="50" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="50" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="51" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="53" t="s">
-        <v>148</v>
-      </c>
-      <c r="D9" s="52" t="s">
+      <c r="D25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="54"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="54"/>
+      <c r="I25" s="54"/>
+    </row>
+    <row r="26" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="B26" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="E9" s="52" t="s">
+      <c r="D26" s="50"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="54"/>
+      <c r="H26" s="54"/>
+      <c r="I26" s="54"/>
+    </row>
+    <row r="27" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="48" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" s="50" t="s">
         <v>162</v>
       </c>
-      <c r="F9" s="52" t="s">
-        <v>163</v>
-      </c>
-      <c r="G9" s="52" t="s">
-        <v>164</v>
-      </c>
-      <c r="H9" s="52" t="s">
-        <v>165</v>
-      </c>
-      <c r="I9" s="52" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="50" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="51" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10" s="54" t="s">
-        <v>167</v>
-      </c>
-      <c r="D10" s="52" t="s">
-        <v>168</v>
-      </c>
-      <c r="E10" s="52" t="s">
-        <v>169</v>
-      </c>
-      <c r="F10" s="52" t="s">
-        <v>170</v>
-      </c>
-      <c r="G10" s="52" t="s">
-        <v>171</v>
-      </c>
-      <c r="H10" s="52" t="s">
-        <v>172</v>
-      </c>
-      <c r="I10" s="52" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="50" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="51" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="55" t="s">
-        <v>174</v>
-      </c>
-      <c r="D11" s="52" t="s">
-        <v>175</v>
-      </c>
-      <c r="E11" s="52" t="s">
-        <v>176</v>
-      </c>
-      <c r="F11" s="52" t="s">
-        <v>177</v>
-      </c>
-      <c r="G11" s="52" t="s">
-        <v>178</v>
-      </c>
-      <c r="H11" s="52" t="s">
-        <v>179</v>
-      </c>
-      <c r="I11" s="52" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="50" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="51" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="D12" s="52" t="s">
-        <v>182</v>
-      </c>
-      <c r="E12" s="52" t="s">
-        <v>176</v>
-      </c>
-      <c r="F12" s="52" t="s">
-        <v>183</v>
-      </c>
-      <c r="G12" s="52" t="s">
-        <v>184</v>
-      </c>
-      <c r="H12" s="52" t="s">
-        <v>185</v>
-      </c>
-      <c r="I12" s="52" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="50" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="D13" s="52" t="s">
-        <v>187</v>
-      </c>
-      <c r="E13" s="52" t="s">
-        <v>176</v>
-      </c>
-      <c r="F13" s="52" t="s">
-        <v>188</v>
-      </c>
-      <c r="G13" s="52" t="s">
-        <v>189</v>
-      </c>
-      <c r="H13" s="52" t="s">
-        <v>190</v>
-      </c>
-      <c r="I13" s="52" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="56" t="s">
-        <v>192</v>
-      </c>
-      <c r="B16" s="56"/>
-      <c r="C16" s="56"/>
-      <c r="D16" s="56"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="56"/>
-      <c r="I16" s="56"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="B19" s="51" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19" s="52" t="s">
-        <v>196</v>
-      </c>
-      <c r="D19" s="52"/>
-      <c r="E19" s="52"/>
-      <c r="F19" s="57"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="57"/>
-      <c r="I19" s="57"/>
-    </row>
-    <row r="20" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="50" t="n">
-        <v>2</v>
-      </c>
-      <c r="B20" s="51" t="s">
-        <v>141</v>
-      </c>
-      <c r="C20" s="52" t="s">
-        <v>197</v>
-      </c>
-      <c r="D20" s="52"/>
-      <c r="E20" s="52"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
-      <c r="H20" s="57"/>
-      <c r="I20" s="57"/>
-    </row>
-    <row r="21" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="50" t="n">
-        <v>3</v>
-      </c>
-      <c r="B21" s="51" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" s="52" t="s">
-        <v>198</v>
-      </c>
-      <c r="D21" s="52"/>
-      <c r="E21" s="52"/>
-      <c r="F21" s="57"/>
-      <c r="G21" s="57"/>
-      <c r="H21" s="57"/>
-      <c r="I21" s="57"/>
-    </row>
-    <row r="22" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="50" t="n">
-        <v>4</v>
-      </c>
-      <c r="B22" s="51" t="s">
-        <v>46</v>
-      </c>
-      <c r="C22" s="52" t="s">
-        <v>199</v>
-      </c>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="57"/>
-      <c r="I22" s="57"/>
-    </row>
-    <row r="23" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="50" t="n">
-        <v>5</v>
-      </c>
-      <c r="B23" s="51" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="52" t="s">
-        <v>200</v>
-      </c>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
-    </row>
-    <row r="24" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="50" t="n">
-        <v>6</v>
-      </c>
-      <c r="B24" s="51" t="s">
-        <v>47</v>
-      </c>
-      <c r="C24" s="52" t="s">
-        <v>201</v>
-      </c>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="57"/>
-      <c r="G24" s="57"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="57"/>
-    </row>
-    <row r="25" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="50" t="n">
-        <v>7</v>
-      </c>
-      <c r="B25" s="51" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="52" t="s">
-        <v>202</v>
-      </c>
-      <c r="D25" s="52"/>
-      <c r="E25" s="52"/>
-      <c r="F25" s="57"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="57"/>
-      <c r="I25" s="57"/>
-    </row>
-    <row r="26" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="50" t="n">
-        <v>8</v>
-      </c>
-      <c r="B26" s="51" t="s">
-        <v>48</v>
-      </c>
-      <c r="C26" s="52" t="s">
-        <v>203</v>
-      </c>
-      <c r="D26" s="52"/>
-      <c r="E26" s="52"/>
-      <c r="F26" s="57"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
-    </row>
-    <row r="27" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="50" t="n">
-        <v>9</v>
-      </c>
-      <c r="B27" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="C27" s="52" t="s">
-        <v>204</v>
-      </c>
-      <c r="D27" s="52"/>
-      <c r="E27" s="52"/>
-      <c r="F27" s="57"/>
-      <c r="G27" s="57"/>
-      <c r="H27" s="57"/>
-      <c r="I27" s="57"/>
+      <c r="D27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="54"/>
+      <c r="G27" s="54"/>
+      <c r="H27" s="54"/>
+      <c r="I27" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -3664,290 +3296,689 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="55" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" s="26" t="n">
+        <v>63000</v>
+      </c>
+      <c r="C5" s="56" t="n">
+        <v>5250</v>
+      </c>
+      <c r="D5" s="57" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>57</v>
+      </c>
+      <c r="F5" s="56" t="n">
+        <v>892417.355521537</v>
+      </c>
+      <c r="G5" s="58" t="s">
+        <v>171</v>
+      </c>
+      <c r="H5" s="58" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="59" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>69000</v>
+      </c>
+      <c r="C6" s="60" t="n">
+        <v>5750</v>
+      </c>
+      <c r="D6" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>57</v>
+      </c>
+      <c r="F6" s="60" t="n">
+        <v>499745.591649637</v>
+      </c>
+      <c r="G6" s="50" t="s">
+        <v>174</v>
+      </c>
+      <c r="H6" s="50" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="59" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>57000</v>
+      </c>
+      <c r="C7" s="60" t="n">
+        <v>4750</v>
+      </c>
+      <c r="D7" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>57</v>
+      </c>
+      <c r="F7" s="60" t="n">
+        <v>1285089.11939344</v>
+      </c>
+      <c r="G7" s="50" t="s">
+        <v>177</v>
+      </c>
+      <c r="H7" s="50" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>63000</v>
+      </c>
+      <c r="C8" s="60" t="n">
+        <v>5250</v>
+      </c>
+      <c r="D8" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>57</v>
+      </c>
+      <c r="F8" s="60" t="n">
+        <v>892417.355521537</v>
+      </c>
+      <c r="G8" s="50" t="s">
+        <v>103</v>
+      </c>
+      <c r="H8" s="50"/>
+    </row>
+    <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="59" t="s">
+        <v>180</v>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>42000</v>
+      </c>
+      <c r="C9" s="60" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D9" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="F9" s="60" t="n">
+        <v>710510.021576641</v>
+      </c>
+      <c r="G9" s="50" t="s">
+        <v>181</v>
+      </c>
+      <c r="H9" s="50" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="59" t="s">
+        <v>183</v>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>78000</v>
+      </c>
+      <c r="C10" s="60" t="n">
+        <v>6500</v>
+      </c>
+      <c r="D10" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>58</v>
+      </c>
+      <c r="F10" s="60" t="n">
+        <v>1017588.10978243</v>
+      </c>
+      <c r="G10" s="50" t="s">
+        <v>184</v>
+      </c>
+      <c r="H10" s="50" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="62" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="63" t="s">
+        <v>187</v>
+      </c>
+      <c r="B14" s="63"/>
+      <c r="C14" s="63"/>
+      <c r="D14" s="63"/>
+      <c r="E14" s="63"/>
+      <c r="F14" s="63"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="63"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="63" t="s">
+        <v>188</v>
+      </c>
+      <c r="B15" s="63"/>
+      <c r="C15" s="63"/>
+      <c r="D15" s="63"/>
+      <c r="E15" s="63"/>
+      <c r="F15" s="63"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="63"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" s="63"/>
+      <c r="C16" s="63"/>
+      <c r="D16" s="63"/>
+      <c r="E16" s="63"/>
+      <c r="F16" s="63"/>
+      <c r="G16" s="63"/>
+      <c r="H16" s="63"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="63" t="s">
+        <v>190</v>
+      </c>
+      <c r="B17" s="63"/>
+      <c r="C17" s="63"/>
+      <c r="D17" s="63"/>
+      <c r="E17" s="63"/>
+      <c r="F17" s="63"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="63"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="63" t="s">
+        <v>191</v>
+      </c>
+      <c r="B18" s="63"/>
+      <c r="C18" s="63"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="63" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" s="63"/>
+      <c r="C19" s="63"/>
+      <c r="D19" s="63"/>
+      <c r="E19" s="63"/>
+      <c r="F19" s="63"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="63"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A19:H19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="64" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="65" t="s">
+        <v>197</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" s="66" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="65" t="s">
+        <v>197</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="C5" s="66" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="65" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="C6" s="66" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="65" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="C7" s="66" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="65" t="s">
+        <v>197</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" s="66" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="65" t="s">
+        <v>203</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="65" t="s">
+        <v>203</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="C10" s="67" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="65" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="C11" s="67" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="65" t="s">
         <v>207</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="13" t="s">
+      <c r="B12" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="13" t="s">
+      <c r="C12" s="8" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="C13" s="8" t="n">
+        <v>58000</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="C14" s="8" t="n">
+        <v>190000</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="58" t="s">
+      <c r="C15" s="8" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="B5" s="59" t="n">
-        <v>57000</v>
-      </c>
-      <c r="C5" s="60" t="n">
-        <v>4750</v>
-      </c>
-      <c r="D5" s="61" t="n">
-        <v>15</v>
-      </c>
-      <c r="E5" s="25" t="n">
-        <v>57</v>
-      </c>
-      <c r="F5" s="60" t="n">
-        <v>1285089.11939344</v>
-      </c>
-      <c r="G5" s="62" t="s">
+      <c r="C16" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="H5" s="62" t="s">
+      <c r="C17" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="63" t="s">
+      <c r="C18" s="8" t="n">
+        <v>473000</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="65" t="s">
         <v>215</v>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>60000</v>
-      </c>
-      <c r="C6" s="64" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D6" s="65" t="n">
-        <v>15</v>
-      </c>
-      <c r="E6" s="15" t="n">
-        <v>57</v>
-      </c>
-      <c r="F6" s="64" t="n">
-        <v>1088753.23745749</v>
-      </c>
-      <c r="G6" s="52" t="s">
+      <c r="B19" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="H6" s="52" t="s">
+      <c r="C19" s="67" t="n">
+        <v>0.07</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="65" t="s">
+        <v>215</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="63" t="s">
+      <c r="C20" s="67" t="n">
+        <v>0.07</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="65" t="s">
+        <v>215</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="B7" s="8" t="n">
-        <v>51000</v>
-      </c>
-      <c r="C7" s="64" t="n">
-        <v>4250</v>
-      </c>
-      <c r="D7" s="65" t="n">
-        <v>14</v>
-      </c>
-      <c r="E7" s="15" t="n">
-        <v>56</v>
-      </c>
-      <c r="F7" s="64" t="n">
-        <v>678282.619881932</v>
-      </c>
-      <c r="G7" s="52" t="s">
+      <c r="C21" s="67" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="65" t="s">
+        <v>215</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="H7" s="52" t="s">
+      <c r="C22" s="67" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="65" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="63" t="s">
+      <c r="B23" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>42000</v>
-      </c>
-      <c r="C8" s="64" t="n">
-        <v>3500</v>
-      </c>
-      <c r="D8" s="65" t="n">
-        <v>13</v>
-      </c>
-      <c r="E8" s="15" t="n">
-        <v>55</v>
-      </c>
-      <c r="F8" s="64" t="n">
-        <v>710510.021576641</v>
-      </c>
-      <c r="G8" s="52" t="s">
+      <c r="C23" s="8" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="65" t="s">
+        <v>220</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="H8" s="52" t="s">
+      <c r="C24" s="8" t="n">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="65" t="s">
+        <v>220</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="63" t="s">
+      <c r="C25" s="8" t="n">
+        <v>8550</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="65" t="s">
+        <v>220</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>66000</v>
-      </c>
-      <c r="C9" s="64" t="n">
-        <v>5500</v>
-      </c>
-      <c r="D9" s="65" t="n">
-        <v>15</v>
-      </c>
-      <c r="E9" s="15" t="n">
-        <v>57</v>
-      </c>
-      <c r="F9" s="64" t="n">
-        <v>696081.473585587</v>
-      </c>
-      <c r="G9" s="52" t="s">
+      <c r="C26" s="8" t="n">
+        <v>2850</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="65" t="s">
+        <v>220</v>
+      </c>
+      <c r="B27" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="H9" s="52" t="s">
+      <c r="C27" s="8" t="n">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="65" t="s">
+        <v>220</v>
+      </c>
+      <c r="B28" s="7" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="66" t="s">
+      <c r="C28" s="8" t="n">
+        <v>42600</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="65" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="67" t="s">
+      <c r="B29" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="B13" s="67"/>
-      <c r="C13" s="67"/>
-      <c r="D13" s="67"/>
-      <c r="E13" s="67"/>
-      <c r="F13" s="67"/>
-      <c r="G13" s="67"/>
-      <c r="H13" s="67"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="67" t="s">
+      <c r="C29" s="66" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="65" t="s">
+        <v>227</v>
+      </c>
+      <c r="B30" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="B14" s="67"/>
-      <c r="C14" s="67"/>
-      <c r="D14" s="67"/>
-      <c r="E14" s="67"/>
-      <c r="F14" s="67"/>
-      <c r="G14" s="67"/>
-      <c r="H14" s="67"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="67" t="s">
+      <c r="C30" s="67" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="65" t="s">
         <v>230</v>
       </c>
-      <c r="B15" s="67"/>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="67"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="67" t="s">
+      <c r="B31" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="B16" s="67"/>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="67"/>
-      <c r="G16" s="67"/>
-      <c r="H16" s="67"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="67" t="s">
+      <c r="C31" s="66" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="65" t="s">
+        <v>230</v>
+      </c>
+      <c r="B32" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="B17" s="67"/>
-      <c r="C17" s="67"/>
-      <c r="D17" s="67"/>
-      <c r="E17" s="67"/>
-      <c r="F17" s="67"/>
-      <c r="G17" s="67"/>
-      <c r="H17" s="67"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="67" t="s">
+      <c r="C32" s="66" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="65" t="s">
         <v>233</v>
       </c>
-      <c r="B18" s="67"/>
-      <c r="C18" s="67"/>
-      <c r="D18" s="67"/>
-      <c r="E18" s="67"/>
-      <c r="F18" s="67"/>
-      <c r="G18" s="67"/>
-      <c r="H18" s="67"/>
+      <c r="B33" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C33" s="67" t="n">
+        <v>0.04</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A18:H18"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3972,21 +4003,21 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="46" t="s">
-        <v>234</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
+      <c r="A1" s="64" t="s">
+        <v>235</v>
+      </c>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4002,28 +4033,28 @@
         <v>4</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4306,100 +4337,100 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="66" t="s">
-        <v>244</v>
+      <c r="A16" s="69" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="69" t="s">
-        <v>245</v>
-      </c>
-      <c r="B17" s="69"/>
-      <c r="C17" s="69"/>
-      <c r="D17" s="69"/>
-      <c r="E17" s="69"/>
-      <c r="F17" s="69"/>
-      <c r="G17" s="69"/>
-      <c r="H17" s="69"/>
-      <c r="I17" s="69"/>
+      <c r="A17" s="70" t="s">
+        <v>246</v>
+      </c>
+      <c r="B17" s="70"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="70"/>
+      <c r="E17" s="70"/>
+      <c r="F17" s="70"/>
+      <c r="G17" s="70"/>
+      <c r="H17" s="70"/>
+      <c r="I17" s="70"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="69" t="s">
-        <v>246</v>
-      </c>
-      <c r="B18" s="69"/>
-      <c r="C18" s="69"/>
-      <c r="D18" s="69"/>
-      <c r="E18" s="69"/>
-      <c r="F18" s="69"/>
-      <c r="G18" s="69"/>
-      <c r="H18" s="69"/>
-      <c r="I18" s="69"/>
+      <c r="A18" s="70" t="s">
+        <v>247</v>
+      </c>
+      <c r="B18" s="70"/>
+      <c r="C18" s="70"/>
+      <c r="D18" s="70"/>
+      <c r="E18" s="70"/>
+      <c r="F18" s="70"/>
+      <c r="G18" s="70"/>
+      <c r="H18" s="70"/>
+      <c r="I18" s="70"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="69" t="s">
-        <v>247</v>
-      </c>
-      <c r="B19" s="69"/>
-      <c r="C19" s="69"/>
-      <c r="D19" s="69"/>
-      <c r="E19" s="69"/>
-      <c r="F19" s="69"/>
-      <c r="G19" s="69"/>
-      <c r="H19" s="69"/>
-      <c r="I19" s="69"/>
+      <c r="A19" s="70" t="s">
+        <v>248</v>
+      </c>
+      <c r="B19" s="70"/>
+      <c r="C19" s="70"/>
+      <c r="D19" s="70"/>
+      <c r="E19" s="70"/>
+      <c r="F19" s="70"/>
+      <c r="G19" s="70"/>
+      <c r="H19" s="70"/>
+      <c r="I19" s="70"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="69" t="s">
-        <v>248</v>
-      </c>
-      <c r="B20" s="69"/>
-      <c r="C20" s="69"/>
-      <c r="D20" s="69"/>
-      <c r="E20" s="69"/>
-      <c r="F20" s="69"/>
-      <c r="G20" s="69"/>
-      <c r="H20" s="69"/>
-      <c r="I20" s="69"/>
+      <c r="A20" s="70" t="s">
+        <v>249</v>
+      </c>
+      <c r="B20" s="70"/>
+      <c r="C20" s="70"/>
+      <c r="D20" s="70"/>
+      <c r="E20" s="70"/>
+      <c r="F20" s="70"/>
+      <c r="G20" s="70"/>
+      <c r="H20" s="70"/>
+      <c r="I20" s="70"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="69" t="s">
-        <v>249</v>
-      </c>
-      <c r="B21" s="69"/>
-      <c r="C21" s="69"/>
-      <c r="D21" s="69"/>
-      <c r="E21" s="69"/>
-      <c r="F21" s="69"/>
-      <c r="G21" s="69"/>
-      <c r="H21" s="69"/>
-      <c r="I21" s="69"/>
+      <c r="A21" s="70" t="s">
+        <v>250</v>
+      </c>
+      <c r="B21" s="70"/>
+      <c r="C21" s="70"/>
+      <c r="D21" s="70"/>
+      <c r="E21" s="70"/>
+      <c r="F21" s="70"/>
+      <c r="G21" s="70"/>
+      <c r="H21" s="70"/>
+      <c r="I21" s="70"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="69" t="s">
-        <v>250</v>
-      </c>
-      <c r="B22" s="69"/>
-      <c r="C22" s="69"/>
-      <c r="D22" s="69"/>
-      <c r="E22" s="69"/>
-      <c r="F22" s="69"/>
-      <c r="G22" s="69"/>
-      <c r="H22" s="69"/>
-      <c r="I22" s="69"/>
+      <c r="A22" s="70" t="s">
+        <v>251</v>
+      </c>
+      <c r="B22" s="70"/>
+      <c r="C22" s="70"/>
+      <c r="D22" s="70"/>
+      <c r="E22" s="70"/>
+      <c r="F22" s="70"/>
+      <c r="G22" s="70"/>
+      <c r="H22" s="70"/>
+      <c r="I22" s="70"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="69" t="s">
-        <v>251</v>
-      </c>
-      <c r="B23" s="69"/>
-      <c r="C23" s="69"/>
-      <c r="D23" s="69"/>
-      <c r="E23" s="69"/>
-      <c r="F23" s="69"/>
-      <c r="G23" s="69"/>
-      <c r="H23" s="69"/>
-      <c r="I23" s="69"/>
+      <c r="A23" s="70" t="s">
+        <v>252</v>
+      </c>
+      <c r="B23" s="70"/>
+      <c r="C23" s="70"/>
+      <c r="D23" s="70"/>
+      <c r="E23" s="70"/>
+      <c r="F23" s="70"/>
+      <c r="G23" s="70"/>
+      <c r="H23" s="70"/>
+      <c r="I23" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -4436,19 +4467,19 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="46" t="s">
-        <v>252</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
+      <c r="A1" s="64" t="s">
+        <v>253</v>
+      </c>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4459,25 +4490,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4725,7 +4756,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>

</xml_diff>